<commit_message>
Batch 1: phones, countries, facets, CLI tests, dead-code removal
- new cleaning_engine/phones.py: formatting normalization (country
  never guessed), implausible lengths flagged; wired into pipeline on
  profile-detected phone columns, all modes
- country names to ISO codes wired in (extended EU map incl. Romanian
  forms); romanian/messy/edge goldens re-frozen after full-column review
- deleted redundant strip_all_strings + semantic-dedupe placeholder
- /api/analyze gains value-frequency facets; frontend renders them (EN/RO)
- CLI tests for clean/analyze; analyzer suggests normalize_phones
- modes table + README cover phones and countries
</commit_message>
<xml_diff>
--- a/cleansheet/tests/fixtures/expected/edge_cases_cleaned.xlsx
+++ b/cleansheet/tests/fixtures/expected/edge_cases_cleaned.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>555-1234</t>
+          <t>5551234</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>555-5678</t>
+          <t>5555678</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>555-9012</t>
+          <t>5559012</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>555-3456</t>
+          <t>5553456</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>555-7890</t>
+          <t>5557890</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>555-1111</t>
+          <t>5551111</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>555-2222</t>
+          <t>5552222</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>555-3333</t>
+          <t>5553333</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>555-4444</t>
+          <t>5554444</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>555-5555</t>
+          <t>5555555</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>555-6666</t>
+          <t>5556666</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>555-7777</t>
+          <t>5557777</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">

</xml_diff>